<commit_message>
update bill page -5560922286
</commit_message>
<xml_diff>
--- a/bills/JXZFSP/-5560922286/a04009deb7e69570bc9f5ca765210e487e41c38d8e120e2341bfe7056a39f72d/bill-2026-06-24.xlsx
+++ b/bills/JXZFSP/-5560922286/a04009deb7e69570bc9f5ca765210e487e41c38d8e120e2341bfe7056a39f72d/bill-2026-06-24.xlsx
@@ -75,183 +75,225 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>06/24 12:36:33</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>180000</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>8.4</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>21428.57</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>马瑞昭</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>tiantiananxin</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t>06/24 12:08:55</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>200000</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>0%</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>8.3</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>24096.39</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>羊美云</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>tiantiananxin</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>代付</t>
-        </is>
-      </c>
-    </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>代付</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>时间</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>金额</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>费率</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>汇率</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>结算</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>标记人</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>操作人</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
       </c>
     </row>
-    <row r="9"/>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>下发</t>
-        </is>
-      </c>
-    </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>下发</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>时间</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>金额</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>标记人</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>操作人</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
       </c>
     </row>
-    <row r="12"/>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>总计</t>
-        </is>
-      </c>
-    </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>总入款</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>200000</t>
+          <t>总计</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>应下发</t>
+          <t>总入款</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>24096.39</t>
+          <t>380000</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>已下发</t>
+          <t>应下发</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>45524.96</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>已下发</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>未下发</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>24096.39</t>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>45524.96</t>
         </is>
       </c>
     </row>

</xml_diff>